<commit_message>
docs: add final verification report and QA evidence
</commit_message>
<xml_diff>
--- a/audit/Aident-verification-report.xlsx
+++ b/audit/Aident-verification-report.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="R6ed6771109454f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="Rbef39f2a7bf34279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Rc968aa5a9f0f40cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="R198ab79ad2ea4992"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="R65e55950c7634379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R8a7fbf64375c4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="Rb5962eca63a546e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="R58a3780f70454d24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Ref87edccf037435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="Re0e1560325e24b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="R3294b25799974aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R5e463c73e2f54563"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1076,11 +1076,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32.88999938964844" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
   </x:cols>
@@ -1128,23 +1128,25 @@
         <x:v>Предварительный одностраничный сайт на подтверждённых данных</x:v>
       </x:c>
       <x:c r="B4" s="31" t="str">
-        <x:v>Белый/чёрный из официального логотипа; акцент задаётся после подбора официальных медиа</x:v>
+        <x:v>Белый/чёрный из официального логотипа</x:v>
       </x:c>
       <x:c r="C4" s="31" t="str">
         <x:v>HTML, CSS, JavaScript</x:v>
       </x:c>
       <x:c r="D4" s="31" t="str">
-        <x:v>Не создан</x:v>
+        <x:v>https://github.com/nuradilabyz/aident-aktau-website-concept</x:v>
       </x:c>
       <x:c r="E4" s="31" t="str">
-        <x:v>Не опубликован</x:v>
+        <x:v>https://nuradilabyz.github.io/aident-aktau-website-concept/</x:v>
       </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>Не выбран</x:v>
-      </x:c>
-      <x:c r="G4" s="31" t="str"/>
+        <x:v>GitHub Pages через GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G4" s="31" t="str">
+        <x:v>14.07.2026</x:v>
+      </x:c>
       <x:c r="H4" s="32" t="str">
-        <x:v>В очереди: отсутствие сайта подтверждено; не использовать WhatsApp и график до уточнения</x:v>
+        <x:v>Опубликован; noindex, nofollow и запрет в robots.txt сохранены до согласования владельцем. WhatsApp и график не опубликованы из-за расхождения источников.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1161,12 +1163,12 @@
   <x:cols>
     <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32.11000061035156" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="28.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -1208,21 +1210,81 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="30" t="str">
-        <x:v>Не применимо</x:v>
-      </x:c>
-      <x:c r="B4" s="31" t="str">
-        <x:v>Не применимо</x:v>
-      </x:c>
-      <x:c r="C4" s="31" t="str"/>
-      <x:c r="D4" s="31" t="str">
-        <x:v>QA не запускался: публичной версии нет</x:v>
-      </x:c>
-      <x:c r="E4" s="31" t="str"/>
-      <x:c r="F4" s="31" t="str"/>
-      <x:c r="G4" s="31" t="str"/>
-      <x:c r="H4" s="32" t="str">
-        <x:v>NOT RUN — публикация запрещена</x:v>
+      <x:c r="A4" s="21" t="str">
+        <x:v>Компьютер</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>1440 px</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>audit/qa-screenshots/desktop-1440-final-hero.png</x:v>
+      </x:c>
+      <x:c r="D4" s="22" t="str">
+        <x:v>Полная страница, hero, контакты и карта; HTTPS; ссылки; консоль; SEO и OG</x:v>
+      </x:c>
+      <x:c r="E4" s="22" t="str">
+        <x:v>В первом проходе найден пустой alt у hero-логотипа</x:v>
+      </x:c>
+      <x:c r="F4" s="22" t="str">
+        <x:v>alt заполнен и опубликован отдельным деплоем</x:v>
+      </x:c>
+      <x:c r="G4" s="22" t="str">
+        <x:v>Повторно проверено на live-версии с cache-busting URL</x:v>
+      </x:c>
+      <x:c r="H4" s="23" t="str">
+        <x:v>QA PASSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="24" t="str">
+        <x:v>Планшет</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="str">
+        <x:v>768 px</x:v>
+      </x:c>
+      <x:c r="C5" s="25" t="str">
+        <x:v>audit/qa-screenshots/tablet-768-final-hero.png</x:v>
+      </x:c>
+      <x:c r="D5" s="25" t="str">
+        <x:v>Адаптив, читаемость, меню, якоря, отсутствие горизонтальной прокрутки</x:v>
+      </x:c>
+      <x:c r="E5" s="25" t="str">
+        <x:v>Нет после исправления</x:v>
+      </x:c>
+      <x:c r="F5" s="25" t="str">
+        <x:v>Не требуется</x:v>
+      </x:c>
+      <x:c r="G5" s="25" t="str">
+        <x:v>Повторно проверено на live-версии</x:v>
+      </x:c>
+      <x:c r="H5" s="26" t="str">
+        <x:v>QA PASSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="27" t="str">
+        <x:v>Мобильный</x:v>
+      </x:c>
+      <x:c r="B6" s="28" t="str">
+        <x:v>390 px</x:v>
+      </x:c>
+      <x:c r="C6" s="28" t="str">
+        <x:v>audit/qa-screenshots/mobile-390-final-hero.png</x:v>
+      </x:c>
+      <x:c r="D6" s="28" t="str">
+        <x:v>Мобильное меню, фиксированная кнопка звонка, ссылки, отображение hero</x:v>
+      </x:c>
+      <x:c r="E6" s="28" t="str">
+        <x:v>Нет после исправления</x:v>
+      </x:c>
+      <x:c r="F6" s="28" t="str">
+        <x:v>Не требуется</x:v>
+      </x:c>
+      <x:c r="G6" s="28" t="str">
+        <x:v>Повторно проверено на live-версии</x:v>
+      </x:c>
+      <x:c r="H6" s="29" t="str">
+        <x:v>QA PASSED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1239,14 +1301,14 @@
   <x:cols>
     <x:col min="1" max="1" width="25.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="30.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -1303,26 +1365,28 @@
         <x:v>+7 775 825 52 43</x:v>
       </x:c>
       <x:c r="C4" s="31" t="str">
-        <x:v>Не использовать до подтверждения номера</x:v>
+        <x:v>Не отправлять до подтверждения номера</x:v>
       </x:c>
       <x:c r="D4" s="31" t="str">
         <x:v>https://www.instagram.com/aident_clinic/</x:v>
       </x:c>
-      <x:c r="E4" s="31" t="str"/>
+      <x:c r="E4" s="31" t="str">
+        <x:v>https://nuradilabyz.github.io/aident-aktau-website-concept/</x:v>
+      </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>Не подготовлено: публичной ссылки ещё нет</x:v>
+        <x:v>Здравствуйте, команда Aident! Подготовил предварительную концепцию сайта для вашей цифровой стоматологии в Актау — с акцентом на коронки, CAD/CAM и 3D-моделирование: https://nuradilabyz.github.io/aident-aktau-website-concept/ Буду рад показать проект и обсудить правки.</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
-        <x:v>Не подготовлено: публичной ссылки ещё нет</x:v>
+        <x:v>Здравствуйте! Подготовил концепцию сайта для Aident с акцентом на цифровые направления. Посмотреть: https://nuradilabyz.github.io/aident-aktau-website-concept/ Могу коротко показать идею и обсудить правки.</x:v>
       </x:c>
       <x:c r="H4" s="31" t="str">
-        <x:v>Не подготовлено: публичной ссылки ещё нет</x:v>
+        <x:v>Здравствуйте! Я подготовил предварительную концепцию сайта Aident на основе 2GIS и официального Instagram. Можно показать ссылку и обсудить, что важно оставить или изменить?</x:v>
       </x:c>
       <x:c r="I4" s="31" t="str">
-        <x:v>Не подготовлено: публичной ссылки ещё нет</x:v>
+        <x:v>Понимаю. Проект ни к чему не обязывает: он показывает, как объединить контакты, 2GIS и цифровые направления клиники. Если сейчас неактуально, можно сохранить ссылку на будущее.</x:v>
       </x:c>
       <x:c r="J4" s="32" t="str">
-        <x:v>Не отправлять</x:v>
+        <x:v>Не отправлять самостоятельно; WhatsApp и график требуют подтверждения владельцем</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: redesign Aident conversion flow
</commit_message>
<xml_diff>
--- a/audit/Aident-verification-report.xlsx
+++ b/audit/Aident-verification-report.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="Rb5962eca63a546e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="R58a3780f70454d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Ref87edccf037435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="Re0e1560325e24b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="R3294b25799974aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R5e463c73e2f54563"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="Rfd636fc74d1940f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="R55e664e4b8d449ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Ra9d2d59e5f124d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="R8ac0f4dca259430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="R968f35c5a29143b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R19444d478c43499e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -631,13 +631,13 @@
         <x:v>WhatsApp</x:v>
       </x:c>
       <x:c r="B7" s="25" t="str">
-        <x:v>Не публиковать до подтверждения владельцем</x:v>
+        <x:v>https://wa.me/77758255243</x:v>
       </x:c>
       <x:c r="C7" s="25" t="str">
-        <x:v>2GIS и Instagram</x:v>
+        <x:v>Карточка 2GIS</x:v>
       </x:c>
       <x:c r="D7" s="26" t="str">
-        <x:v>РАСХОЖДЕНИЕ: 2GIS ведёт на wa.me/77758255243, а ссылка в bio Instagram — wa.me/7758255243</x:v>
+        <x:v>Использован как CTA в обновлённой концепции по запросу пользователя; требуется подтверждение владельцем, поскольку bio Instagram ведёт на wa.me/7758255243</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -701,13 +701,13 @@
         <x:v>Отзывы</x:v>
       </x:c>
       <x:c r="B12" s="25" t="str">
-        <x:v>13 текстовых отзывов; 36 оценок</x:v>
+        <x:v>Рейтинг 4.9; в концепции использованы два коротких публичных фрагмента</x:v>
       </x:c>
       <x:c r="C12" s="25" t="str">
         <x:v>https://2gis.kz/aktau/firm/70000001028449496/tab/reviews</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
-        <x:v>Наблюдение 14.07.2026; число оценок может меняться</x:v>
+        <x:v>Наблюдение 14.07.2026; число оценок сознательно не публикуется и может меняться</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -763,7 +763,7 @@
         <x:v>Публичные источники проверены</x:v>
       </x:c>
       <x:c r="D16" s="29" t="str">
-        <x:v>Не подтверждено для сайта</x:v>
+        <x:v>Не подтверждены имена, специализации и согласие на использование фото; раздел врачей исключён</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -848,7 +848,7 @@
         <x:v>Каталог / карта</x:v>
       </x:c>
       <x:c r="F4" s="33" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G4" s="33" t="str">
         <x:v>audit/screenshots/web/2gis-contacts.webp</x:v>
@@ -877,7 +877,7 @@
         <x:v>Официальная социальная сеть</x:v>
       </x:c>
       <x:c r="F5" s="35" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G5" s="35" t="str">
         <x:v>audit/screenshots/web/instagram-profile-header.webp</x:v>
@@ -906,7 +906,7 @@
         <x:v>Поиск / каталоги / соцсети</x:v>
       </x:c>
       <x:c r="F6" s="35" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G6" s="35" t="str">
         <x:v>Не применимо</x:v>
@@ -929,7 +929,7 @@
       <x:c r="D7" s="37" t="str"/>
       <x:c r="E7" s="37" t="str"/>
       <x:c r="F7" s="37" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G7" s="37" t="str"/>
       <x:c r="H7" s="37" t="str">
@@ -954,8 +954,8 @@
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32.11000061035156" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="19.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
   </x:cols>
@@ -1011,7 +1011,7 @@
         <x:v>2GIS</x:v>
       </x:c>
       <x:c r="F4" s="22" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G4" s="23" t="str">
         <x:v>Оптимизированная публичная копия контактов; не является медиа для сайта.</x:v>
@@ -1034,33 +1034,79 @@
         <x:v>aident_clinic</x:v>
       </x:c>
       <x:c r="F5" s="25" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
+        <x:v>2026-07-14 12:15 +05:00</x:v>
       </x:c>
       <x:c r="G5" s="26" t="str">
         <x:v>Оптимизированная копия заголовка профиля, логотипа, bio, ссылки WhatsApp и контактной кнопки; персональная навигация пользователя не попала в кадр.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="27" t="str">
+      <x:c r="A6" s="24" t="str">
         <x:v>Логотип</x:v>
       </x:c>
-      <x:c r="B6" s="28" t="str">
+      <x:c r="B6" s="25" t="str">
         <x:v>media/logo/aident-instagram-avatar.jpg</x:v>
       </x:c>
-      <x:c r="C6" s="28" t="str">
+      <x:c r="C6" s="25" t="str">
         <x:v>https://www.instagram.com/aident_clinic/</x:v>
       </x:c>
-      <x:c r="D6" s="28" t="str">
+      <x:c r="D6" s="25" t="str">
         <x:v>Планируется: шапка, favicon, Open Graph</x:v>
       </x:c>
-      <x:c r="E6" s="28" t="str">
+      <x:c r="E6" s="25" t="str">
         <x:v>aident_clinic</x:v>
       </x:c>
-      <x:c r="F6" s="28" t="str">
-        <x:v>2026-07-14 02:09 +05:00</x:v>
-      </x:c>
-      <x:c r="G6" s="29" t="str">
+      <x:c r="F6" s="25" t="str">
+        <x:v>2026-07-14 12:15 +05:00</x:v>
+      </x:c>
+      <x:c r="G6" s="26" t="str">
         <x:v>Официальный аватар профиля, публично получен через страницу, 1080×1080; пропорции не изменены.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="24" t="str">
+        <x:v>Отзывы</x:v>
+      </x:c>
+      <x:c r="B7" s="25" t="str">
+        <x:v>Нет локального медиа</x:v>
+      </x:c>
+      <x:c r="C7" s="25" t="str">
+        <x:v>https://2gis.kz/aktau/firm/70000001028449496/tab/reviews</x:v>
+      </x:c>
+      <x:c r="D7" s="25" t="str">
+        <x:v>Раздел отзывов</x:v>
+      </x:c>
+      <x:c r="E7" s="25" t="str">
+        <x:v>2GIS; публичные авторы отзывов</x:v>
+      </x:c>
+      <x:c r="F7" s="25" t="str">
+        <x:v>2026-07-14 12:15 +05:00</x:v>
+      </x:c>
+      <x:c r="G7" s="26" t="str">
+        <x:v>Использованы только короткие цитаты: «Золотые руки и трепетное отношение» (Margarita Zholdasova) и «Отличная клиника!» (Exxon M).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>Карта</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="str">
+        <x:v>site/assets/media/map/aident-2gis-map.png</x:v>
+      </x:c>
+      <x:c r="C8" s="28" t="str">
+        <x:v>https://beautyshare.2gis.ru/api/v1/image?city=aktau&amp;zoom=17&amp;center=51.164119%2C43.668692&amp;title=Aident&amp;desc=28-%D0%B9%20%D0%BC%D0%B8%D0%BA%D1%80%D0%BE%D1%80%D0%B0%D0%B9%D0%BE%D0%BD%2C%201%2C%20%D0%90%D0%BA%D1%82%D0%B0%D1%83</x:v>
+      </x:c>
+      <x:c r="D8" s="28" t="str">
+        <x:v>Блок контактов; ссылка на карточку 2GIS</x:v>
+      </x:c>
+      <x:c r="E8" s="28" t="str">
+        <x:v>2GIS</x:v>
+      </x:c>
+      <x:c r="F8" s="28" t="str">
+        <x:v>2026-07-14 12:15 +05:00</x:v>
+      </x:c>
+      <x:c r="G8" s="29" t="str">
+        <x:v>Публичный статичный превью-слой 2GIS с точкой Aident; не используется Google Maps.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1076,7 +1122,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
@@ -1125,10 +1171,10 @@
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="30" t="str">
-        <x:v>Предварительный одностраничный сайт на подтверждённых данных</x:v>
+        <x:v>Предварительный одностраничный сайт: выбор услуг, о клинике, отзывы 2GIS, карта 2GIS и запись в WhatsApp</x:v>
       </x:c>
       <x:c r="B4" s="31" t="str">
-        <x:v>Белый/чёрный из официального логотипа</x:v>
+        <x:v>Чёрный/белый логотип; тёплый нейтральный интерфейс</x:v>
       </x:c>
       <x:c r="C4" s="31" t="str">
         <x:v>HTML, CSS, JavaScript</x:v>
@@ -1146,7 +1192,7 @@
         <x:v>14.07.2026</x:v>
       </x:c>
       <x:c r="H4" s="32" t="str">
-        <x:v>Опубликован; noindex, nofollow и запрет в robots.txt сохранены до согласования владельцем. WhatsApp и график не опубликованы из-за расхождения источников.</x:v>
+        <x:v>Обновление подготовлено к деплою. noindex, nofollow и запрет в robots.txt сохранены. WhatsApp взят из 2GIS и ждёт подтверждения владельцем; график не опубликован.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1301,7 +1347,7 @@
   <x:cols>
     <x:col min="1" max="1" width="25.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="30.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
@@ -1365,7 +1411,7 @@
         <x:v>+7 775 825 52 43</x:v>
       </x:c>
       <x:c r="C4" s="31" t="str">
-        <x:v>Не отправлять до подтверждения номера</x:v>
+        <x:v>https://wa.me/77758255243 (требует подтверждения владельцем)</x:v>
       </x:c>
       <x:c r="D4" s="31" t="str">
         <x:v>https://www.instagram.com/aident_clinic/</x:v>
@@ -1374,19 +1420,19 @@
         <x:v>https://nuradilabyz.github.io/aident-aktau-website-concept/</x:v>
       </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>Здравствуйте, команда Aident! Подготовил предварительную концепцию сайта для вашей цифровой стоматологии в Актау — с акцентом на коронки, CAD/CAM и 3D-моделирование: https://nuradilabyz.github.io/aident-aktau-website-concept/ Буду рад показать проект и обсудить правки.</x:v>
+        <x:v>Здравствуйте, команда Aident! Подготовил предварительную концепцию сайта для вашей цифровой стоматологии в Актау — с выбором услуг, короткими отзывами из 2GIS и маршрутом 2GIS: https://nuradilabyz.github.io/aident-aktau-website-concept/ Буду рад показать проект и обсудить правки.</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
-        <x:v>Здравствуйте! Подготовил концепцию сайта для Aident с акцентом на цифровые направления. Посмотреть: https://nuradilabyz.github.io/aident-aktau-website-concept/ Могу коротко показать идею и обсудить правки.</x:v>
+        <x:v>Здравствуйте! Подготовил концепцию сайта для Aident с услугами, 2GIS и WhatsApp-записью. Посмотреть: https://nuradilabyz.github.io/aident-aktau-website-concept/ Могу коротко показать идею и обсудить правки.</x:v>
       </x:c>
       <x:c r="H4" s="31" t="str">
         <x:v>Здравствуйте! Я подготовил предварительную концепцию сайта Aident на основе 2GIS и официального Instagram. Можно показать ссылку и обсудить, что важно оставить или изменить?</x:v>
       </x:c>
       <x:c r="I4" s="31" t="str">
-        <x:v>Понимаю. Проект ни к чему не обязывает: он показывает, как объединить контакты, 2GIS и цифровые направления клиники. Если сейчас неактуально, можно сохранить ссылку на будущее.</x:v>
+        <x:v>Понимаю. Проект ни к чему не обязывает: он показывает, как объединить запись в WhatsApp, 2GIS и цифровые направления клиники. Если сейчас неактуально, можно сохранить ссылку на будущее.</x:v>
       </x:c>
       <x:c r="J4" s="32" t="str">
-        <x:v>Не отправлять самостоятельно; WhatsApp и график требуют подтверждения владельцем</x:v>
+        <x:v>Не отправлять самостоятельно; номер WhatsApp и график требуют подтверждения владельцем</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: add redesign QA evidence
</commit_message>
<xml_diff>
--- a/audit/Aident-verification-report.xlsx
+++ b/audit/Aident-verification-report.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="Rfd636fc74d1940f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="R55e664e4b8d449ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Ra9d2d59e5f124d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="R8ac0f4dca259430c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="R968f35c5a29143b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R19444d478c43499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clinic Data" sheetId="1" r:id="Rbcbff0bceea2450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Verification" sheetId="2" r:id="R8e5761b450da48e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Media" sheetId="3" r:id="Rf40d5ba57d4b48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Website Production" sheetId="4" r:id="R5d858171afd645fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Report" sheetId="5" r:id="Rb797af7e16a54717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="6" r:id="R86e746fa5f494590"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1192,7 +1192,7 @@
         <x:v>14.07.2026</x:v>
       </x:c>
       <x:c r="H4" s="32" t="str">
-        <x:v>Обновление подготовлено к деплою. noindex, nofollow и запрет в robots.txt сохранены. WhatsApp взят из 2GIS и ждёт подтверждения владельцем; график не опубликован.</x:v>
+        <x:v>Опубликовано и повторно проверено QA. noindex, nofollow и запрет в robots.txt сохранены. WhatsApp взят из 2GIS и ждёт подтверждения владельцем; график не опубликован.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1263,19 +1263,19 @@
         <x:v>1440 px</x:v>
       </x:c>
       <x:c r="C4" s="22" t="str">
-        <x:v>audit/qa-screenshots/desktop-1440-final-hero.png</x:v>
+        <x:v>audit/qa-screenshots/redesign-recheck-1440-full.png; redesign-recheck-1440-contacts-map.png</x:v>
       </x:c>
       <x:c r="D4" s="22" t="str">
-        <x:v>Полная страница, hero, контакты и карта; HTTPS; ссылки; консоль; SEO и OG</x:v>
+        <x:v>Полная страница, hero, услуги, отзывы, контакты и карта; HTTPS; ссылки; console; SEO и OG</x:v>
       </x:c>
       <x:c r="E4" s="22" t="str">
-        <x:v>В первом проходе найден пустой alt у hero-логотипа</x:v>
+        <x:v>На первом проходе карта 2GIS была чрезмерно затемнена — география читалась плохо</x:v>
       </x:c>
       <x:c r="F4" s="22" t="str">
-        <x:v>alt заполнен и опубликован отдельным деплоем</x:v>
+        <x:v>Ослаблено overlay-затемнение; CTA маршрута получила отдельную контрастную подложку; опубликован новый CSS URL</x:v>
       </x:c>
       <x:c r="G4" s="22" t="str">
-        <x:v>Повторно проверено на live-версии с cache-busting URL</x:v>
+        <x:v>Повторно проверено на live-версии ?qa=map-fix-20260714: улицы, точка Aident, адрес и CTA читаемы</x:v>
       </x:c>
       <x:c r="H4" s="23" t="str">
         <x:v>QA PASSED</x:v>
@@ -1289,10 +1289,10 @@
         <x:v>768 px</x:v>
       </x:c>
       <x:c r="C5" s="25" t="str">
-        <x:v>audit/qa-screenshots/tablet-768-final-hero.png</x:v>
+        <x:v>audit/qa-screenshots/redesign-recheck-768-full.png</x:v>
       </x:c>
       <x:c r="D5" s="25" t="str">
-        <x:v>Адаптив, читаемость, меню, якоря, отсутствие горизонтальной прокрутки</x:v>
+        <x:v>Полная страница; hero, услуги, отзывы, контакты; отсутствие горизонтальной прокрутки и ошибок консоли</x:v>
       </x:c>
       <x:c r="E5" s="25" t="str">
         <x:v>Нет после исправления</x:v>
@@ -1301,7 +1301,7 @@
         <x:v>Не требуется</x:v>
       </x:c>
       <x:c r="G5" s="25" t="str">
-        <x:v>Повторно проверено на live-версии</x:v>
+        <x:v>На live-версии 753 px контента ≤ 768 px viewport; console []</x:v>
       </x:c>
       <x:c r="H5" s="26" t="str">
         <x:v>QA PASSED</x:v>
@@ -1315,10 +1315,10 @@
         <x:v>390 px</x:v>
       </x:c>
       <x:c r="C6" s="28" t="str">
-        <x:v>audit/qa-screenshots/mobile-390-final-hero.png</x:v>
+        <x:v>audit/qa-screenshots/redesign-recheck-390-full.png; redesign-recheck-390-menu-open.png; redesign-recheck-390-contacts-map.png; redesign-recheck-390-map-lower-sticky.png</x:v>
       </x:c>
       <x:c r="D6" s="28" t="str">
-        <x:v>Мобильное меню, фиксированная кнопка звонка, ссылки, отображение hero</x:v>
+        <x:v>Полная страница, hero, услуги, отзывы, мобильное меню, фиксированная WhatsApp-кнопка, карта и нижняя область</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
         <x:v>Нет после исправления</x:v>
@@ -1327,7 +1327,7 @@
         <x:v>Не требуется</x:v>
       </x:c>
       <x:c r="G6" s="28" t="str">
-        <x:v>Повторно проверено на live-версии</x:v>
+        <x:v>На live-версии 375 px контента ≤ 390 px viewport; меню aria-expanded=true; CTA не закрывает кнопку карты</x:v>
       </x:c>
       <x:c r="H6" s="29" t="str">
         <x:v>QA PASSED</x:v>

</xml_diff>